<commit_message>
Stjernekort: opdater DVR-testdata med Udbudsbetingelser + rettede kilder
Tilføjer Udbudsbetingelser + Tilbudsbrev + Bilag A/B til DVR-testdata,
svarende til ESDH-strukturen. Bilag 5 og Bilag 12 er opdateret med rigtige
rettelser fra det virkelige materiale: Bilag 5 citerer nu korrekt
"Kontraktens punkt 23.2" (var 24.2), og Bilag 12 citerer nu korrekt "bilag
5, punkt 7.4" (var 8.4) - begge de tidligere kendte DVR-fejl er dermed
rettet ved kilden, jf. tests/test_dvr.py::test_ingen_brudte_henvisninger.

De to samlede QA-notater er fjernet, da testdata/dvr-mappen i mellemtiden
er blevet erstattet med et nyt, komplet sæt (og de tilhørende filer derfor
ikke længere findes).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Stjernekort/testdata/dvr/24. Bilag 12_Leverancevederlag og betalingsplan samt øvrige priser_Appendiks A_Prisskema.xlsx
+++ b/Stjernekort/testdata/dvr/24. Bilag 12_Leverancevederlag og betalingsplan samt øvrige priser_Appendiks A_Prisskema.xlsx
@@ -8242,8 +8242,8 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x01010024373CE2A0AAA344A185260442135A2D" ma:contentTypeVersion="7" ma:contentTypeDescription="Opret et nyt dokument." ma:contentTypeScope="" ma:versionID="76ad4519aa1714fde3c96c2403e508d7">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2a4fc43e-74cb-4ecd-8f0b-7e4e11483b0c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="62d884777905cb7988e89b8e230839d6" ns2:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010024373CE2A0AAA344A185260442135A2D" ma:contentTypeVersion="7" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c352957fb64d73ea37153bc8851dd08b">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2a4fc43e-74cb-4ecd-8f0b-7e4e11483b0c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cdc15103199d3093eb4a2dfc161609bd" ns2:_="">
     <xsd:import namespace="2a4fc43e-74cb-4ecd-8f0b-7e4e11483b0c"/>
     <xsd:element name="properties">
       <xsd:complexType>
@@ -8317,8 +8317,8 @@
         <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Indholdstype"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Titel"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
         <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
         <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
@@ -8419,13 +8419,13 @@
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
-    <Godkendtafkunden xmlns="2a4fc43e-74cb-4ecd-8f0b-7e4e11483b0c">Udestår</Godkendtafkunden>
+    <Godkendtafkunden xmlns="2a4fc43e-74cb-4ecd-8f0b-7e4e11483b0c">Klar til upload</Godkendtafkunden>
   </documentManagement>
 </p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3DCC35C2-7B68-4E5C-BBA0-DB5C4A20AD47}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{11CEE5DB-3D97-4C0F-B6D6-FAD00B42A349}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>